<commit_message>
samples: demonstrate template image movement
</commit_message>
<xml_diff>
--- a/samples/fixed_range_charts_output.xlsx
+++ b/samples/fixed_range_charts_output.xlsx
@@ -596,84 +596,84 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>3</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="6480000" cy="3240000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="6480000" cy="3240000"/>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm/>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>26</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="6480000" cy="3240000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="6480000" cy="3240000"/>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm/>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>26</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="6480000" cy="3240000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="6480000" cy="3240000"/>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm/>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>